<commit_message>
Dash Hedge IPCA - 2026-03-03
</commit_message>
<xml_diff>
--- a/Dados/ativos_mapeados_com_taxa_efetiva.xlsx
+++ b/Dados/ativos_mapeados_com_taxa_efetiva.xlsx
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1.062938081797936</v>
+        <v>1.062862511354904</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.031649836844364</v>
+        <v>1.031621464981925</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1.031649836844364</v>
+        <v>1.031621464981925</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1.026691004408933</v>
+        <v>1.0266637404173</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1.026691004408933</v>
+        <v>1.0266637404173</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.023681210689404</v>
+        <v>1.023669954692576</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2125,7 +2125,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1.052488639161389</v>
+        <v>1.052487262760346</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1.052488639161389</v>
+        <v>1.052487262760346</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1.052488639161389</v>
+        <v>1.052487262760346</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1.015984776187372</v>
+        <v>1.015982556066905</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>1.013470243265679</v>
+        <v>1.011717717542436</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -3145,7 +3145,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.013470243265679</v>
+        <v>1.011717717542436</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>1.015991948917102</v>
+        <v>1.015989988663004</v>
       </c>
       <c r="I64" t="inlineStr">
         <is>
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>1.015991948917102</v>
+        <v>1.015989988663004</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>1.050625</v>
+        <v>1.050497965289035</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
@@ -3549,7 +3549,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1.050625</v>
+        <v>1.050497965289035</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>1.064997093019325</v>
+        <v>1.064916450955605</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>1.062938081797936</v>
+        <v>1.062862511354904</v>
       </c>
       <c r="I84" t="inlineStr">
         <is>
@@ -4221,7 +4221,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>1.062938081797936</v>
+        <v>1.062862511354904</v>
       </c>
       <c r="I85" t="inlineStr">
         <is>
@@ -4269,7 +4269,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>1.062938081797936</v>
+        <v>1.062862511354904</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
@@ -4413,7 +4413,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>1.144518010602442</v>
+        <v>1.144378917056012</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -4461,7 +4461,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>1.144518010602442</v>
+        <v>1.144378917056012</v>
       </c>
       <c r="I90" t="inlineStr">
         <is>
@@ -4509,7 +4509,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>1.144518010602442</v>
+        <v>1.144378917056012</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Dash DI - 2026-07-13
</commit_message>
<xml_diff>
--- a/Dados/ativos_mapeados_com_taxa_efetiva.xlsx
+++ b/Dados/ativos_mapeados_com_taxa_efetiva.xlsx
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1.016679840302595</v>
+        <v>1.016511732460023</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1.016679840302595</v>
+        <v>1.016511732460023</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1.016679840302595</v>
+        <v>1.016511732460023</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1.058550815989044</v>
+        <v>1.035313360558953</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1.058550815989044</v>
+        <v>1.035313360558953</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1.04537937504615</v>
+        <v>1.035313360558953</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J10" t="b">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1.032479330249586</v>
+        <v>1.032476523828006</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.032479330249586</v>
+        <v>1.032476523828006</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1.032479330249586</v>
+        <v>1.032476523828006</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1.032479330249586</v>
+        <v>1.032476523828006</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1.032479330249586</v>
+        <v>1.032476523828006</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1.032479330249586</v>
+        <v>1.032476523828006</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1269,7 +1269,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1.027481208289491</v>
+        <v>1.0274786630262</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1.027481208289491</v>
+        <v>1.0274786630262</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>1.312943</v>
+        <v>1.307094</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1541,7 +1541,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>1.312943</v>
+        <v>1.307094</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>1.031817</v>
+        <v>1.030641</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>1.031817</v>
+        <v>1.030641</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1.031817</v>
+        <v>1.030641</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.031817</v>
+        <v>1.030641</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.031817</v>
+        <v>1.030641</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1.052138784815274</v>
+        <v>1.046169955658442</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1.052138784815274</v>
+        <v>1.046169955658442</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>1.052138784815274</v>
+        <v>1.046169955658442</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -2349,11 +2349,11 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>1.02858992832202</v>
+        <v>1.046169955658442</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J43" t="b">
@@ -3141,7 +3141,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1.016226620178901</v>
+        <v>1.016085755815899</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -3225,7 +3225,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>1.016226620178901</v>
+        <v>1.016085755815899</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>1.020749</v>
+        <v>1.020018</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -3401,7 +3401,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>1.020749</v>
+        <v>1.020018</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
@@ -3537,7 +3537,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1.016379649932376</v>
+        <v>1.016302694975625</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -3761,7 +3761,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>1.043402160663369</v>
+        <v>1.04296980890625</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>1.043402160663369</v>
+        <v>1.04296980890625</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
@@ -4029,7 +4029,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>1.060074022977964</v>
+        <v>1.059747868494567</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>1.058550815989044</v>
+        <v>1.035313360558953</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>1.058550815989044</v>
+        <v>1.035313360558953</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -4609,7 +4609,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>1.058550815989044</v>
+        <v>1.035313360558953</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -4753,7 +4753,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>1.137748629076882</v>
+        <v>1.07740539991251</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
@@ -4801,7 +4801,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>1.137748629076882</v>
+        <v>1.07740539991251</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>1.137748629076882</v>
+        <v>1.07740539991251</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Dash DI - 02/09/2026
</commit_message>
<xml_diff>
--- a/Dados/ativos_mapeados_com_taxa_efetiva.xlsx
+++ b/Dados/ativos_mapeados_com_taxa_efetiva.xlsx
@@ -601,11 +601,11 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1.0569</v>
+        <v>1.02</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J4" t="b">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1.034885761650082</v>
+        <v>1.034712084469143</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1.034885761650082</v>
+        <v>1.034712084469143</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1.04537937504615</v>
+        <v>1.0252348601965</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -777,7 +777,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1.04537937504615</v>
+        <v>1.0252348601965</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1.04537937504615</v>
+        <v>1.0252348601965</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1.034885761650082</v>
+        <v>1.034712084469143</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1.034885761650082</v>
+        <v>1.034712084469143</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1.032449941153846</v>
+        <v>1.03239988471142</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1.032449941153846</v>
+        <v>1.03239988471142</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1.032449941153846</v>
+        <v>1.03239988471142</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1.032449941153846</v>
+        <v>1.03239988471142</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1.032449941153846</v>
+        <v>1.03239988471142</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1.032449941153846</v>
+        <v>1.03239988471142</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>1.027455331736998</v>
+        <v>1.027414900915792</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1361,11 +1361,11 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1.06</v>
+        <v>1.027414900915792</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J21" t="b">
@@ -1405,11 +1405,11 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1.06</v>
+        <v>1.027414900915792</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J22" t="b">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1.027455331736998</v>
+        <v>1.027414900915792</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1540,12 +1540,10 @@
           <t>2026-07-10 00:00:00</t>
         </is>
       </c>
-      <c r="H25" t="n">
-        <v>1.307094</v>
-      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J25" t="b">
@@ -1588,16 +1586,14 @@
           <t>2026-07-10 00:00:00</t>
         </is>
       </c>
-      <c r="H26" t="n">
-        <v>1.307094</v>
-      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="J26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1633,7 +1629,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>1.030641</v>
+        <v>1.028614</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1677,7 +1673,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1.030641</v>
+        <v>1.028614</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1721,7 +1717,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1.030641</v>
+        <v>1.028614</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1765,7 +1761,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1.030641</v>
+        <v>1.029422</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1813,7 +1809,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>1.030641</v>
+        <v>1.028614</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2037,11 +2033,11 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1.02858992832202</v>
+        <v>1.035</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J36" t="b">
@@ -2081,11 +2077,11 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>1.02858992832202</v>
+        <v>1.035</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J37" t="b">
@@ -2125,11 +2121,11 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>1.02858992832202</v>
+        <v>1.035</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J38" t="b">
@@ -2169,11 +2165,11 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>1.02858992832202</v>
+        <v>1.035</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J39" t="b">
@@ -2213,11 +2209,11 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>1.02858992832202</v>
+        <v>1.035</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J40" t="b">
@@ -2441,7 +2437,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2529,7 +2525,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -3145,7 +3141,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>0.00399851</v>
+        <v>0.00373305</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -3357,11 +3353,11 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>1.020018</v>
+        <v>1.003</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J66" t="b">
@@ -3449,11 +3445,11 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>1.020018</v>
+        <v>1.003</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J68" t="b">
@@ -3493,11 +3489,11 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>1.012998</v>
+        <v>1.003</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J69" t="b">
@@ -3537,11 +3533,11 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1.012998</v>
+        <v>1.003</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>ISIN</t>
+          <t>MATRIZ</t>
         </is>
       </c>
       <c r="J70" t="b">
@@ -3585,7 +3581,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>1.012219553815679</v>
+        <v>1.003</v>
       </c>
       <c r="I71" t="inlineStr">
         <is>
@@ -3629,7 +3625,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>0.00399851</v>
+        <v>0.00373305</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
@@ -3673,7 +3669,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>1.021813</v>
+        <v>1.016004</v>
       </c>
       <c r="I73" t="inlineStr">
         <is>
@@ -3717,7 +3713,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>1.027364</v>
+        <v>1.021813</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -3761,7 +3757,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>1.035107</v>
+        <v>1.032555</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -3809,7 +3805,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>1.044027056767213</v>
+        <v>1.04236373705509</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
@@ -3853,7 +3849,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>1.044027056767213</v>
+        <v>1.04236373705509</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
@@ -3897,7 +3893,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>1.035107</v>
+        <v>1.032555</v>
       </c>
       <c r="I78" t="inlineStr">
         <is>
@@ -3941,7 +3937,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>1.049916</v>
+        <v>1.048077</v>
       </c>
       <c r="I79" t="inlineStr">
         <is>
@@ -3985,7 +3981,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>1.049916</v>
+        <v>1.049006</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
@@ -4029,7 +4025,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>1.049916</v>
+        <v>1.048077</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -4077,7 +4073,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>1.060596901321775</v>
+        <v>1.059268852932506</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
@@ -4121,7 +4117,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>1.049916</v>
+        <v>1.048077</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -4513,7 +4509,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>1.087205</v>
+        <v>1.08453</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
@@ -4561,7 +4557,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>1.034885761650082</v>
+        <v>1.034712084469143</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -4609,7 +4605,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>1.034885761650082</v>
+        <v>1.034712084469143</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -4657,7 +4653,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>1.034885761650082</v>
+        <v>1.034712084469143</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -4801,7 +4797,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>1.07045790198874</v>
+        <v>1.069664153441496</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
@@ -4849,7 +4845,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>1.07045790198874</v>
+        <v>1.069664153441496</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
@@ -4897,7 +4893,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>1.07045790198874</v>
+        <v>1.069664153441496</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>

</xml_diff>